<commit_message>
fix(clase-01): correct 2026 tariff and add PPTX slide generator
Fixes same tariff errors (factor 1.13213) found in clase-02 source:
- tablas-comparativas.md: annual brackets 8-11 and monthly brackets 8-11
  corrected; carga efectiva examples recalculated
- ejercicios-practicos.md: Ejercicio 2C ($180K sueldo) fixed from
  ISR $47,993 (wrong bracket 32%) to $50,304 (correct bracket 34%);
  UMA/SMG header values updated to match clase-02 standards
- ejercicios-excel/generate.py: TARIFA_MENSUAL_2026 and TARIFA_ANUAL_2026
  corrected; Excel files regenerated

Adds generate_slides.py: produces slides-clase-01-modulo-04.pptx from
slides-scripts.md extracting only Contenido Visual (no instructor scripts).
Applies TodoConta design system (#0B5FFF · #0A1628 · #FAFAF7 · Inter).

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/modulo-04-isr-personas-fisicas/clase-01-regimenes-fiscales-pf/ejercicios-excel/01-retencion-isr-mensual.xlsx
+++ b/modulo-04-isr-personas-fisicas/clase-01-regimenes-fiscales-pf/ejercicios-excel/01-retencion-isr-mensual.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Instrucciones" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Datos" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Ejercicio" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Solución" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Datos" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ejercicio" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Solución" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -897,7 +897,7 @@
         <v>55640.59</v>
       </c>
       <c r="C12" s="7" t="n">
-        <v>167424.91</v>
+        <v>106410.49</v>
       </c>
       <c r="D12" s="7" t="n">
         <v>10434.61</v>
@@ -911,13 +911,13 @@
         <v>9</v>
       </c>
       <c r="B13" s="7" t="n">
-        <v>167424.92</v>
+        <v>106410.5</v>
       </c>
       <c r="C13" s="7" t="n">
-        <v>223233.22</v>
+        <v>141880.67</v>
       </c>
       <c r="D13" s="7" t="n">
-        <v>43969.91</v>
+        <v>25666.64</v>
       </c>
       <c r="E13" s="8" t="n">
         <v>0.32</v>
@@ -928,13 +928,13 @@
         <v>10</v>
       </c>
       <c r="B14" s="7" t="n">
-        <v>223233.23</v>
+        <v>141880.68</v>
       </c>
       <c r="C14" s="7" t="n">
-        <v>669699.66</v>
+        <v>425643.66</v>
       </c>
       <c r="D14" s="7" t="n">
-        <v>61828.55</v>
+        <v>37344.33</v>
       </c>
       <c r="E14" s="8" t="n">
         <v>0.34</v>
@@ -945,13 +945,13 @@
         <v>11</v>
       </c>
       <c r="B15" s="7" t="n">
-        <v>669699.67</v>
+        <v>425643.67</v>
       </c>
       <c r="C15" s="7" t="n">
         <v>999999999.99</v>
       </c>
       <c r="D15" s="7" t="n">
-        <v>213619.92</v>
+        <v>133897.59</v>
       </c>
       <c r="E15" s="8" t="n">
         <v>0.35</v>

</xml_diff>